<commit_message>
1.2.4.3 Projects step 1: Projects names in export and import; SalesTeam Excel export/import (one workbook, accounts + contacts + projects); CRM exports always both files; all-or-filtered asked for every filter; one Leads Export; Resolve Web Findings moved to Settings; Export opens at once
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/code/Target_Accounts_Template.xlsx
+++ b/code/Target_Accounts_Template.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Companies" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Contacts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Initiatives" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Projects" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Investment" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sources" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Exclusion_List" sheetId="6" state="visible" r:id="rId6"/>
@@ -407,7 +407,7 @@
     </comment>
     <comment ref="AT1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Short text list of the main relevant initiatives</t>
+        <t>Optional. Short text list of the main relevant projects</t>
       </text>
     </comment>
     <comment ref="AU1" authorId="0" shapeId="0">
@@ -577,7 +577,7 @@
   <commentList>
     <comment ref="A1" authorId="0" shapeId="0">
       <text>
-        <t>MANDATORY. Unique initiative ID</t>
+        <t>MANDATORY. Unique project ID</t>
       </text>
     </comment>
     <comment ref="B1" authorId="0" shapeId="0">
@@ -592,7 +592,7 @@
     </comment>
     <comment ref="D1" authorId="0" shapeId="0">
       <text>
-        <t>MANDATORY. Short name of the initiative</t>
+        <t>MANDATORY. Short name of the project</t>
       </text>
     </comment>
     <comment ref="E1" authorId="0" shapeId="0">
@@ -617,7 +617,7 @@
     </comment>
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Stage of the initiative, e.g. Pilot, Production, Scaling</t>
+        <t>Optional. Stage of the project, e.g. Pilot, Production, Scaling</t>
       </text>
     </comment>
     <comment ref="J1" authorId="0" shapeId="0">
@@ -1211,7 +1211,7 @@
     <col width="21" customWidth="1" min="43" max="43"/>
     <col width="19" customWidth="1" min="44" max="44"/>
     <col width="25" customWidth="1" min="45" max="45"/>
-    <col width="19" customWidth="1" min="46" max="46"/>
+    <col width="16" customWidth="1" min="46" max="46"/>
     <col width="27" customWidth="1" min="47" max="47"/>
     <col width="23" customWidth="1" min="48" max="48"/>
     <col width="28" customWidth="1" min="49" max="49"/>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="AT1" s="2" t="inlineStr">
         <is>
-          <t>Top_Initiatives</t>
+          <t>Top_Projects</t>
         </is>
       </c>
       <c r="AU1" s="2" t="inlineStr">
@@ -1673,10 +1673,10 @@
   <dimension ref="A1:P1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
@@ -1694,7 +1694,7 @@
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Initiative_ID</t>
+          <t>Project_ID</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -1709,7 +1709,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Initiative_Name</t>
+          <t>Project_Name</t>
         </is>
       </c>
       <c r="E1" s="2" t="inlineStr">
@@ -2145,7 +2145,7 @@
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>A Companies sheet with a Company column (one row per account). Add Company_ID to link Contacts, Initiatives, Investment, Sources and Aliases to their company.</t>
+          <t>A Companies sheet with a Company column (one row per account). Add Company_ID to link Contacts, Projects, Investment, Sources and Aliases to their company.</t>
         </is>
       </c>
     </row>
@@ -2176,7 +2176,7 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Initiatives: Initiative_ID, Company_ID, Company, Initiative_Name</t>
+          <t>Projects: Project_ID, Company_ID, Company, Project_Name</t>
         </is>
       </c>
     </row>

</xml_diff>